<commit_message>
Update all places affected by the circuit simplifaction
</commit_message>
<xml_diff>
--- a/docs/05-Power-Budget/PowerBudget_ZiceSun.xlsx
+++ b/docs/05-Power-Budget/PowerBudget_ZiceSun.xlsx
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1 (Zice Sun, 2026-10-16)</t>
+          <t>2 (Zice Sun, 2026-10-26: MCP6004 removed per instructor feedback)</t>
         </is>
       </c>
       <c r="C5" s="76" t="n"/>
@@ -1164,24 +1164,24 @@
       <c r="A11" s="99" t="n"/>
       <c r="B11" s="79" t="inlineStr">
         <is>
-          <t>Quad op amp (low-pass filter)</t>
+          <t>Load cell (bridge excitation)</t>
         </is>
       </c>
       <c r="C11" s="79" t="inlineStr">
         <is>
-          <t>MCP6004-I/P</t>
+          <t>3135_0 (Phidgets)</t>
         </is>
       </c>
       <c r="D11" s="81" t="inlineStr">
         <is>
-          <t>1.8 - 6.0 V</t>
+          <t>5 V max</t>
         </is>
       </c>
       <c r="E11" s="81" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="82" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G11" s="83">
         <f>E11*F11</f>
@@ -1195,27 +1195,11 @@
     </row>
     <row r="12" ht="30" customHeight="1" s="75">
       <c r="A12" s="99" t="n"/>
-      <c r="B12" s="85" t="inlineStr">
-        <is>
-          <t>Load cell (bridge excitation)</t>
-        </is>
-      </c>
-      <c r="C12" s="85" t="inlineStr">
-        <is>
-          <t>3135_0 (Phidgets)</t>
-        </is>
-      </c>
-      <c r="D12" s="86" t="inlineStr">
-        <is>
-          <t>5 V max</t>
-        </is>
-      </c>
-      <c r="E12" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="87" t="n">
-        <v>5</v>
-      </c>
+      <c r="B12" s="85" t="n"/>
+      <c r="C12" s="85" t="n"/>
+      <c r="D12" s="86" t="n"/>
+      <c r="E12" s="80" t="n"/>
+      <c r="F12" s="87" t="n"/>
       <c r="G12" s="83">
         <f>E12*F12</f>
         <v/>
@@ -1321,12 +1305,12 @@
     </row>
     <row r="18" ht="30" customHeight="1" s="75">
       <c r="A18" s="99" t="n"/>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>None on this board</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1339,7 +1323,7 @@
       <c r="E18" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="0" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="70">
@@ -1633,24 +1617,24 @@
       <c r="A32" s="99" t="n"/>
       <c r="B32" s="79" t="inlineStr">
         <is>
-          <t>Quad op amp (low-pass filter)</t>
+          <t>Load cell (bridge excitation)</t>
         </is>
       </c>
       <c r="C32" s="79" t="inlineStr">
         <is>
-          <t>MCP6004-I/P</t>
+          <t>3135_0 (Phidgets)</t>
         </is>
       </c>
       <c r="D32" s="81" t="inlineStr">
         <is>
-          <t>1.8 - 6.0 V</t>
+          <t>5 V max</t>
         </is>
       </c>
       <c r="E32" s="81" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="82" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="G32" s="83">
         <f>E32*F32</f>
@@ -1664,27 +1648,11 @@
     </row>
     <row r="33" ht="30" customHeight="1" s="75">
       <c r="A33" s="99" t="n"/>
-      <c r="B33" s="79" t="inlineStr">
-        <is>
-          <t>Load cell (bridge excitation)</t>
-        </is>
-      </c>
-      <c r="C33" s="79" t="inlineStr">
-        <is>
-          <t>3135_0 (Phidgets)</t>
-        </is>
-      </c>
-      <c r="D33" s="81" t="inlineStr">
-        <is>
-          <t>5 V max</t>
-        </is>
-      </c>
-      <c r="E33" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="82" t="n">
-        <v>5</v>
-      </c>
+      <c r="B33" s="79" t="n"/>
+      <c r="C33" s="79" t="n"/>
+      <c r="D33" s="81" t="n"/>
+      <c r="E33" s="81" t="n"/>
+      <c r="F33" s="82" t="n"/>
       <c r="G33" s="83">
         <f>E33*F33</f>
         <v/>
@@ -1875,7 +1843,7 @@
       <c r="A42" s="99" t="n"/>
       <c r="B42" s="85" t="inlineStr">
         <is>
-          <t>None: all op amps are single-supply</t>
+          <t>None: every part is single-supply</t>
         </is>
       </c>
       <c r="C42" s="79" t="inlineStr">
@@ -2115,7 +2083,7 @@
           <t>None on this board</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2128,7 +2096,7 @@
       <c r="E53" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F53" t="n">
+      <c r="F53" s="0" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="70">
@@ -2512,7 +2480,7 @@
           <t>+3.3V regulator (not used)</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2525,7 +2493,7 @@
       <c r="E72" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="F72" t="n">
+      <c r="F72" s="0" t="n">
         <v>0</v>
       </c>
       <c r="G72" s="70">
@@ -2793,12 +2761,12 @@
     </row>
     <row r="85" ht="30" customHeight="1" s="75">
       <c r="A85" s="99" t="n"/>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="0" t="inlineStr">
         <is>
           <t>No battery (wall-powered board)</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="0" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2861,14 +2829,14 @@
     <row r="90" ht="46" customHeight="1" s="75">
       <c r="A90" s="103" t="inlineStr">
         <is>
-          <t>Absolute maximum currents are worst-case datasheet limits: PIC18F57Q43 maximum current on VDD pin 350 mA (48-pin device, -40 to +85 C); INA125P quiescent current 0.525 mA max plus 12 mA output short-circuit current; MCP6004 30 mA maximum current at supply pins; load cell 5 V excitation across its 1 kOhm bridge = 5 mA.</t>
+          <t>Absolute maximum currents are worst-case datasheet limits: PIC18F57Q43 maximum current on VDD pin 350 mA (48-pin device, -40 to +85 C); INA125P quiescent current 0.525 mA max plus 12 mA output short-circuit current; load cell 5 V excitation across its 1 kOhm bridge = 5 mA. The MCP6004 was removed: the INA125P alone sets the gain and a passive RC filter (no current draw) replaces the active filter.</t>
         </is>
       </c>
     </row>
     <row r="91" ht="46" customHeight="1" s="75">
       <c r="A91" s="103" t="inlineStr">
         <is>
-          <t>Worst-case L7805ABV-DG dissipation: (9 V - 5 V) x 497 mA = 2.0 W, so the regulator gets a Boyd 507302B00000G TO-220 heatsink. Expected normal draw is under 100 mA (about 0.4 W).</t>
+          <t>Worst-case L7805ABV-DG dissipation: (9 V - 5 V) x 459 mA = 1.8 W, so the regulator gets a Boyd 507302B00000G TO-220 heatsink. Expected normal draw is under 100 mA (about 0.4 W).</t>
         </is>
       </c>
     </row>

</xml_diff>